<commit_message>
use the gpu partition
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_gpu.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_gpu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dcl3nd\dev\TRITON-SWMM_toolkit\test_data\norfolk_coastal_flooding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECDD1BC4-26A2-4D5A-82E7-60712843CB3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A04AED4-55EF-4BFF-BE5E-4925170A333F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="15">
   <si>
     <t>hardware_utilization_strategy</t>
   </si>
@@ -75,9 +75,6 @@
   </si>
   <si>
     <t>mem_gb_per_cpu</t>
-  </si>
-  <si>
-    <t>gpu-a6000</t>
   </si>
   <si>
     <t>Use</t>
@@ -713,7 +710,7 @@
         <v>10</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -739,7 +736,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I2" s="11">
         <v>8</v>
@@ -784,7 +781,7 @@
         <v>5</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I3" s="11">
         <v>8</v>
@@ -829,7 +826,7 @@
         <v>6</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I4" s="11">
         <v>8</v>
@@ -874,7 +871,7 @@
         <v>7</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I5" s="11">
         <v>8</v>
@@ -919,7 +916,7 @@
         <v>8</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I6" s="11">
         <v>8</v>
@@ -964,7 +961,7 @@
         <v>16</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I7" s="11">
         <v>8</v>

</xml_diff>

<commit_message>
include 2 gpu job
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_gpu.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_gpu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dcl3nd\dev\TRITON-SWMM_toolkit\test_data\norfolk_coastal_flooding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A04AED4-55EF-4BFF-BE5E-4925170A333F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B463C042-9BC9-4E5C-B5C3-045FE75CCF2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="15">
   <si>
     <t>hardware_utilization_strategy</t>
   </si>
@@ -343,10 +343,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:M7" totalsRowShown="0">
-  <autoFilter ref="A1:M7" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M7">
-    <sortCondition ref="M1:M7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:M8" totalsRowShown="0">
+  <autoFilter ref="A1:M8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M8">
+    <sortCondition ref="M1:M8"/>
   </sortState>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="hardware_utilization_strategy"/>
@@ -655,7 +655,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.85546875" style="14" bestFit="1" customWidth="1"/>
@@ -772,13 +772,13 @@
         <v>1</v>
       </c>
       <c r="E3" s="10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F3" s="10">
         <v>1</v>
       </c>
       <c r="G3" s="10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H3" s="11" t="s">
         <v>12</v>
@@ -788,15 +788,15 @@
       </c>
       <c r="J3" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K3" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L3" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M3" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -817,13 +817,13 @@
         <v>1</v>
       </c>
       <c r="E4" s="10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F4" s="10">
         <v>1</v>
       </c>
       <c r="G4" s="10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H4" s="11" t="s">
         <v>12</v>
@@ -833,15 +833,15 @@
       </c>
       <c r="J4" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K4" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L4" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M4" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -862,13 +862,13 @@
         <v>1</v>
       </c>
       <c r="E5" s="10">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F5" s="10">
         <v>1</v>
       </c>
       <c r="G5" s="10">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>12</v>
@@ -878,15 +878,15 @@
       </c>
       <c r="J5" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K5" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L5" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M5" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -907,13 +907,13 @@
         <v>1</v>
       </c>
       <c r="E6" s="10">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F6" s="10">
         <v>1</v>
       </c>
       <c r="G6" s="10">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>12</v>
@@ -923,15 +923,15 @@
       </c>
       <c r="J6" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K6" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L6" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M6" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -949,16 +949,16 @@
         <v>12</v>
       </c>
       <c r="D7" s="10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="10">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F7" s="10">
         <v>1</v>
       </c>
       <c r="G7" s="10">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H7" s="11" t="s">
         <v>12</v>
@@ -968,17 +968,62 @@
       </c>
       <c r="J7" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="K7" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="L7" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>8</v>
       </c>
       <c r="M7" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="10">
+        <v>2</v>
+      </c>
+      <c r="E8" s="10">
+        <v>16</v>
+      </c>
+      <c r="F8" s="10">
+        <v>1</v>
+      </c>
+      <c r="G8" s="10">
+        <v>16</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" s="11">
+        <v>8</v>
+      </c>
+      <c r="J8" s="12">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
+      </c>
+      <c r="K8" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>16</v>
+      </c>
+      <c r="L8" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="M8" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
test 1, 2, and 5 gpus
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_gpu.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_gpu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dcl3nd\dev\TRITON-SWMM_toolkit\test_data\norfolk_coastal_flooding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B463C042-9BC9-4E5C-B5C3-045FE75CCF2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BBECF4-A6AD-43F1-9B4E-8CD32042767C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2580" yWindow="2550" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="15">
   <si>
     <t>hardware_utilization_strategy</t>
   </si>
@@ -343,10 +343,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:M8" totalsRowShown="0">
-  <autoFilter ref="A1:M8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M8">
-    <sortCondition ref="M1:M8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:M4" totalsRowShown="0">
+  <autoFilter ref="A1:M4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M4">
+    <sortCondition ref="M1:M4"/>
   </sortState>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="hardware_utilization_strategy"/>
@@ -655,7 +655,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.85546875" style="14" bestFit="1" customWidth="1"/>
@@ -848,186 +848,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="10">
-        <v>1</v>
-      </c>
-      <c r="E5" s="10">
-        <v>6</v>
-      </c>
-      <c r="F5" s="10">
-        <v>1</v>
-      </c>
-      <c r="G5" s="10">
-        <v>6</v>
-      </c>
-      <c r="H5" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="11">
-        <v>8</v>
-      </c>
-      <c r="J5" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>6</v>
-      </c>
-      <c r="K5" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>6</v>
-      </c>
-      <c r="L5" s="13">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>6</v>
-      </c>
-      <c r="M5" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="10">
-        <v>1</v>
-      </c>
-      <c r="E6" s="10">
-        <v>7</v>
-      </c>
-      <c r="F6" s="10">
-        <v>1</v>
-      </c>
-      <c r="G6" s="10">
-        <v>7</v>
-      </c>
-      <c r="H6" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" s="11">
-        <v>8</v>
-      </c>
-      <c r="J6" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>7</v>
-      </c>
-      <c r="K6" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>7</v>
-      </c>
-      <c r="L6" s="13">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>7</v>
-      </c>
-      <c r="M6" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="10">
-        <v>1</v>
-      </c>
-      <c r="E7" s="10">
-        <v>8</v>
-      </c>
-      <c r="F7" s="10">
-        <v>1</v>
-      </c>
-      <c r="G7" s="10">
-        <v>8</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" s="11">
-        <v>8</v>
-      </c>
-      <c r="J7" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
-      </c>
-      <c r="K7" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
-      </c>
-      <c r="L7" s="13">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
-      </c>
-      <c r="M7" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="10">
-        <v>2</v>
-      </c>
-      <c r="E8" s="10">
-        <v>16</v>
-      </c>
-      <c r="F8" s="10">
-        <v>1</v>
-      </c>
-      <c r="G8" s="10">
-        <v>16</v>
-      </c>
-      <c r="H8" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I8" s="11">
-        <v>8</v>
-      </c>
-      <c r="J8" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
-      </c>
-      <c r="K8" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
-      </c>
-      <c r="L8" s="13">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
-      </c>
-      <c r="M8" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
run full test gpu sweep on UVA
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_gpu.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_gpu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dcl3nd\dev\TRITON-SWMM_toolkit\test_data\norfolk_coastal_flooding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BBECF4-A6AD-43F1-9B4E-8CD32042767C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{71339603-BCB1-42FF-8601-E4EED22A167E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2580" yWindow="2550" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="15">
   <si>
     <t>hardware_utilization_strategy</t>
   </si>
@@ -343,10 +343,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:M4" totalsRowShown="0">
-  <autoFilter ref="A1:M4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M4">
-    <sortCondition ref="M1:M4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:M8" totalsRowShown="0">
+  <autoFilter ref="A1:M8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M8">
+    <sortCondition ref="M1:M8"/>
   </sortState>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="hardware_utilization_strategy"/>
@@ -655,7 +655,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.85546875" style="14" bestFit="1" customWidth="1"/>
@@ -848,6 +848,186 @@
         <v>1</v>
       </c>
     </row>
+    <row r="5" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="10">
+        <v>1</v>
+      </c>
+      <c r="E5" s="10">
+        <v>6</v>
+      </c>
+      <c r="F5" s="10">
+        <v>1</v>
+      </c>
+      <c r="G5" s="10">
+        <v>6</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" s="11">
+        <v>8</v>
+      </c>
+      <c r="J5" s="12">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>6</v>
+      </c>
+      <c r="K5" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>6</v>
+      </c>
+      <c r="L5" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>6</v>
+      </c>
+      <c r="M5" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="10">
+        <v>1</v>
+      </c>
+      <c r="E6" s="10">
+        <v>7</v>
+      </c>
+      <c r="F6" s="10">
+        <v>1</v>
+      </c>
+      <c r="G6" s="10">
+        <v>7</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="11">
+        <v>8</v>
+      </c>
+      <c r="J6" s="12">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>7</v>
+      </c>
+      <c r="K6" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>7</v>
+      </c>
+      <c r="L6" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>7</v>
+      </c>
+      <c r="M6" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="10">
+        <v>1</v>
+      </c>
+      <c r="E7" s="10">
+        <v>8</v>
+      </c>
+      <c r="F7" s="10">
+        <v>1</v>
+      </c>
+      <c r="G7" s="10">
+        <v>8</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="11">
+        <v>8</v>
+      </c>
+      <c r="J7" s="12">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
+      </c>
+      <c r="K7" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>8</v>
+      </c>
+      <c r="L7" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="M7" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="10">
+        <v>2</v>
+      </c>
+      <c r="E8" s="10">
+        <v>16</v>
+      </c>
+      <c r="F8" s="10">
+        <v>1</v>
+      </c>
+      <c r="G8" s="10">
+        <v>16</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" s="11">
+        <v>8</v>
+      </c>
+      <c r="J8" s="12">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
+      </c>
+      <c r="K8" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>16</v>
+      </c>
+      <c r="L8" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="M8" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
targeted multi gpu testing
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_gpu.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_gpu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dcl3nd\dev\TRITON-SWMM_toolkit\test_data\norfolk_coastal_flooding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{71339603-BCB1-42FF-8601-E4EED22A167E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AB5F63B-1FFA-415E-AFAF-ACF7D8F44D63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2580" yWindow="2550" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="15">
   <si>
     <t>hardware_utilization_strategy</t>
   </si>
@@ -118,7 +118,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -140,8 +140,14 @@
         <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -229,11 +235,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC6C6C6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFC6C6C6"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -281,6 +326,30 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -343,10 +412,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:M8" totalsRowShown="0">
-  <autoFilter ref="A1:M8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M8">
-    <sortCondition ref="M1:M8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:M7" totalsRowShown="0">
+  <autoFilter ref="A1:M7" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M6">
+    <sortCondition ref="M1:M6"/>
   </sortState>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="hardware_utilization_strategy"/>
@@ -655,7 +724,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.85546875" style="14" bestFit="1" customWidth="1"/>
@@ -862,13 +931,13 @@
         <v>1</v>
       </c>
       <c r="E5" s="10">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F5" s="10">
         <v>1</v>
       </c>
       <c r="G5" s="10">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>12</v>
@@ -878,15 +947,15 @@
       </c>
       <c r="J5" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K5" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L5" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M5" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -904,16 +973,16 @@
         <v>12</v>
       </c>
       <c r="D6" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" s="10">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F6" s="10">
         <v>1</v>
       </c>
       <c r="G6" s="10">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>12</v>
@@ -923,107 +992,62 @@
       </c>
       <c r="J6" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K6" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L6" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M6" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="10">
-        <v>1</v>
-      </c>
-      <c r="E7" s="10">
-        <v>8</v>
-      </c>
-      <c r="F7" s="10">
-        <v>1</v>
-      </c>
-      <c r="G7" s="10">
-        <v>8</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" s="11">
-        <v>8</v>
-      </c>
-      <c r="J7" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
-      </c>
-      <c r="K7" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
-      </c>
-      <c r="L7" s="13">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
-      </c>
-      <c r="M7" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="10">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="20">
         <v>2</v>
       </c>
-      <c r="E8" s="10">
+      <c r="E7" s="20">
         <v>16</v>
       </c>
-      <c r="F8" s="10">
-        <v>1</v>
-      </c>
-      <c r="G8" s="10">
+      <c r="F7" s="20">
+        <v>1</v>
+      </c>
+      <c r="G7" s="20">
         <v>16</v>
       </c>
-      <c r="H8" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I8" s="11">
-        <v>8</v>
-      </c>
-      <c r="J8" s="12">
+      <c r="H7" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="22">
+        <v>8</v>
+      </c>
+      <c r="J7" s="23">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>16</v>
       </c>
-      <c r="K8" s="12">
+      <c r="K7" s="23">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>16</v>
       </c>
-      <c r="L8" s="13">
+      <c r="L7" s="24">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>8</v>
       </c>
-      <c r="M8" t="b">
+      <c r="M7" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
         <v>1</v>
       </c>

</xml_diff>